<commit_message>
Field records dataset: acres column, weights derived from yield; update chapter, workbook, script outputs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod03_field_records_cleaning.xlsx
+++ b/textbook_examples/mod03_field_records_cleaning.xlsx
@@ -447,7 +447,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Source: field_records_messy.csv -- one season of spring wheat field records, constructed to contain the eight data-quality issues from Module 3.</t>
+          <t>Source: field_records_messy.csv -- one season of spring wheat field records, constructed to contain the eight data-quality issues from Module 3. Harvest weights are consistent with yield x acres, so the columns can be checked against each other.</t>
         </is>
       </c>
     </row>
@@ -502,35 +502,35 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Text in a numeric column    -- harvest weight unit stripped in Clean column E</t>
+          <t xml:space="preserve">  2. Text in a numeric column    -- harvest weight unit stripped in Clean column F</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Duplicate rows              -- counted on Checks; flagged in Clean column H</t>
+          <t xml:space="preserve">  3. Duplicate rows              -- counted on Checks; flagged in Clean column I</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. Missing-value codes         -- -99, N/A, missing, 9999 blanked in Clean columns D and G</t>
+          <t xml:space="preserve">  4. Missing-value codes         -- -99, N/A, missing, 9999 blanked in Clean columns E and H</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5. Impossible values           -- the -12 and 1250 yields blanked in Clean column D</t>
+          <t xml:space="preserve">  5. Impossible values           -- the -12 and 1250 yields blanked in Clean column E</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  6. Mixed units                 -- N rates below 1 converted from t/ha to kg/ha in Clean column F</t>
+          <t xml:space="preserve">  6. Mixed units                 -- N rates below 1 converted from t/ha to kg/ha in Clean column G</t>
         </is>
       </c>
     </row>
@@ -559,16 +559,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,20 +590,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Acres</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Yield (bu/ac)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>harvest weight</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>N rate</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Moisture %</t>
         </is>
@@ -625,18 +631,21 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>230.3 t</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>118.6</v>
+        <v>160</v>
+      </c>
+      <c r="E2" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>297.7 t</t>
+        </is>
       </c>
       <c r="G2" t="n">
-        <v>15.5</v>
+        <v>97.09999999999999</v>
+      </c>
+      <c r="H2" t="n">
+        <v>12.4</v>
       </c>
     </row>
     <row r="3">
@@ -656,18 +665,21 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>60</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>169.4 t</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>95.5</v>
+        <v>320</v>
+      </c>
+      <c r="E3" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>476.0 t</t>
+        </is>
       </c>
       <c r="G3" t="n">
-        <v>12.4</v>
+        <v>96.2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>14.7</v>
       </c>
     </row>
     <row r="4">
@@ -683,22 +695,25 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026/05/14</t>
+          <t>2026/06/04</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>60.3</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>128.8 t</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>0.125</v>
+        <v>120</v>
+      </c>
+      <c r="E4" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>172.6 t</t>
+        </is>
       </c>
       <c r="G4" t="n">
-        <v>13.7</v>
+        <v>0.081</v>
+      </c>
+      <c r="H4" t="n">
+        <v>12.3</v>
       </c>
     </row>
     <row r="5">
@@ -714,22 +729,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>May-23-2026</t>
+          <t>Jun-18-2026</t>
         </is>
       </c>
       <c r="D5" t="n">
+        <v>320</v>
+      </c>
+      <c r="E5" t="n">
         <v>-99</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>174.2 t</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>134.3</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>642.5 t</t>
+        </is>
       </c>
       <c r="G5" t="n">
-        <v>13.8</v>
+        <v>116.7</v>
+      </c>
+      <c r="H5" t="n">
+        <v>15.4</v>
       </c>
     </row>
     <row r="6">
@@ -745,22 +763,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>05-19-2026</t>
+          <t>06-06-2026</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>118.6 t</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>137.2</v>
+        <v>320</v>
+      </c>
+      <c r="E6" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>561.5 t</t>
+        </is>
       </c>
       <c r="G6" t="n">
-        <v>14.4</v>
+        <v>89.90000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12.3</v>
       </c>
     </row>
     <row r="7">
@@ -776,21 +797,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>115.8 t</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="G7" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="E7" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>222.8 t</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -809,22 +833,25 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026/05/24</t>
+          <t>2026/06/07</t>
         </is>
       </c>
       <c r="D8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E8" t="n">
         <v>-12</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>216.6 t</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>140.9</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>138.6 t</t>
+        </is>
       </c>
       <c r="G8" t="n">
-        <v>15</v>
+        <v>135.9</v>
+      </c>
+      <c r="H8" t="n">
+        <v>14.5</v>
       </c>
     </row>
     <row r="9">
@@ -840,22 +867,25 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>May-02-2026</t>
+          <t>May-18-2026</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>63.7</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>102.8 t</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>91.8</v>
+        <v>160</v>
+      </c>
+      <c r="E9" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>264.0 t</t>
+        </is>
       </c>
       <c r="G9" t="n">
-        <v>15.5</v>
+        <v>127.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>12.4</v>
       </c>
     </row>
     <row r="10">
@@ -871,22 +901,25 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>05-18-2026</t>
+          <t>05-20-2026</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>97.4 t</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>0.134</v>
+        <v>160</v>
+      </c>
+      <c r="E10" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>226.5 t</t>
+        </is>
       </c>
       <c r="G10" t="n">
-        <v>14.5</v>
+        <v>0.081</v>
+      </c>
+      <c r="H10" t="n">
+        <v>13.7</v>
       </c>
     </row>
     <row r="11">
@@ -902,22 +935,25 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>214.6 t</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
+        <v>160</v>
+      </c>
+      <c r="E11" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>256.6 t</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="G11" t="n">
-        <v>14.3</v>
+      <c r="H11" t="n">
+        <v>16.4</v>
       </c>
     </row>
     <row r="12">
@@ -933,22 +969,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026/06/15</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>235.8 t</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>104</v>
+        <v>320</v>
+      </c>
+      <c r="E12" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>481.3 t</t>
+        </is>
       </c>
       <c r="G12" t="n">
-        <v>15.8</v>
+        <v>82.90000000000001</v>
+      </c>
+      <c r="H12" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -964,22 +1003,25 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>May-07-2026</t>
+          <t>May-17-2026</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>182.9 t</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>0.127</v>
+        <v>240</v>
+      </c>
+      <c r="E13" t="n">
+        <v>62</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>402.2 t</t>
+        </is>
       </c>
       <c r="G13" t="n">
-        <v>13.3</v>
+        <v>0.103</v>
+      </c>
+      <c r="H13" t="n">
+        <v>13.5</v>
       </c>
     </row>
     <row r="14">
@@ -995,22 +1037,25 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>05-14-2026</t>
+          <t>05-18-2026</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>58.2</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>107.1 t</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>102.2</v>
+        <v>240</v>
+      </c>
+      <c r="E14" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>269.8 t</t>
+        </is>
       </c>
       <c r="G14" t="n">
-        <v>14</v>
+        <v>82.7</v>
+      </c>
+      <c r="H14" t="n">
+        <v>16.5</v>
       </c>
     </row>
     <row r="15">
@@ -1026,21 +1071,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>176.8 t</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>128.6</v>
-      </c>
-      <c r="G15" t="inlineStr">
+        <v>160</v>
+      </c>
+      <c r="E15" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>249.6 t</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>134</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1059,22 +1107,25 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026/05/18</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>130.2 t</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
+        <v>160</v>
+      </c>
+      <c r="E16" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>234.9 t</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
         <v>0.106</v>
       </c>
-      <c r="G16" t="n">
-        <v>14.5</v>
+      <c r="H16" t="n">
+        <v>11.6</v>
       </c>
     </row>
     <row r="17">
@@ -1090,22 +1141,25 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>May-20-2026</t>
+          <t>May-17-2026</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>240.8 t</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>103.2</v>
+        <v>160</v>
+      </c>
+      <c r="E17" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>225.5 t</t>
+        </is>
       </c>
       <c r="G17" t="n">
-        <v>15.7</v>
+        <v>128.5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="18">
@@ -1125,17 +1179,20 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>179.5 t</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>113.7</v>
+        <v>240</v>
+      </c>
+      <c r="E18" t="n">
+        <v>63</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>418.7 t</t>
+        </is>
       </c>
       <c r="G18" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="H18" t="n">
         <v>15.5</v>
       </c>
     </row>
@@ -1152,22 +1209,25 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>73.8</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>114.6 t</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>0.141</v>
+        <v>160</v>
+      </c>
+      <c r="E19" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>283.2 t</t>
+        </is>
       </c>
       <c r="G19" t="n">
-        <v>12.4</v>
+        <v>0.112</v>
+      </c>
+      <c r="H19" t="n">
+        <v>15.7</v>
       </c>
     </row>
     <row r="20">
@@ -1187,18 +1247,21 @@
         </is>
       </c>
       <c r="D20" t="n">
+        <v>120</v>
+      </c>
+      <c r="E20" t="n">
         <v>1250</v>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>200.4 t</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>138</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>177.8 t</t>
+        </is>
       </c>
       <c r="G20" t="n">
-        <v>13.8</v>
+        <v>104.1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>12.6</v>
       </c>
     </row>
     <row r="21">
@@ -1214,22 +1277,25 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Jun-27-2026</t>
+          <t>Jun-11-2026</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>143.5 t</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>140.1</v>
+        <v>160</v>
+      </c>
+      <c r="E21" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>323.9 t</t>
+        </is>
       </c>
       <c r="G21" t="n">
-        <v>13.3</v>
+        <v>84.7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>13.1</v>
       </c>
     </row>
     <row r="22">
@@ -1245,22 +1311,25 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>05-15-2026</t>
+          <t>06-10-2026</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>71</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>201.3 t</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>0.101</v>
+        <v>240</v>
+      </c>
+      <c r="E22" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>431.7 t</t>
+        </is>
       </c>
       <c r="G22" t="n">
-        <v>14.7</v>
+        <v>0.129</v>
+      </c>
+      <c r="H22" t="n">
+        <v>15.4</v>
       </c>
     </row>
     <row r="23">
@@ -1276,21 +1345,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>68.3</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>253.9 t</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>320</v>
+      </c>
+      <c r="E23" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>492.0 t</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1305,22 +1377,25 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026/05/03</t>
+          <t>2026/05/09</t>
         </is>
       </c>
       <c r="D24" t="n">
+        <v>240</v>
+      </c>
+      <c r="E24" t="n">
         <v>-99</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>140.5 t</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>130.3</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>365.8 t</t>
+        </is>
       </c>
       <c r="G24" t="n">
-        <v>13.6</v>
+        <v>87.2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="25">
@@ -1336,22 +1411,25 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Jun-11-2026</t>
+          <t>Jun-26-2026</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>61.3</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>187.9 t</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>0.111</v>
+        <v>120</v>
+      </c>
+      <c r="E25" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>150.5 t</t>
+        </is>
       </c>
       <c r="G25" t="n">
-        <v>15.8</v>
+        <v>0.124</v>
+      </c>
+      <c r="H25" t="n">
+        <v>15.3</v>
       </c>
     </row>
     <row r="26">
@@ -1367,22 +1445,25 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-10-2026</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>146.0 t</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>134</v>
+        <v>160</v>
+      </c>
+      <c r="E26" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>226.1 t</t>
+        </is>
       </c>
       <c r="G26" t="n">
-        <v>12.8</v>
+        <v>100.8</v>
+      </c>
+      <c r="H26" t="n">
+        <v>11.6</v>
       </c>
     </row>
     <row r="27">
@@ -1398,22 +1479,25 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>124.4 t</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>140.6</v>
+        <v>160</v>
+      </c>
+      <c r="E27" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>252.7 t</t>
+        </is>
       </c>
       <c r="G27" t="n">
-        <v>16.3</v>
+        <v>132.9</v>
+      </c>
+      <c r="H27" t="n">
+        <v>15.7</v>
       </c>
     </row>
     <row r="28">
@@ -1429,22 +1513,25 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026/05/13</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>60</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>206.4 t</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>0.129</v>
+        <v>80</v>
+      </c>
+      <c r="E28" t="n">
+        <v>54</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>120.3 t</t>
+        </is>
       </c>
       <c r="G28" t="n">
-        <v>15.6</v>
+        <v>0.13</v>
+      </c>
+      <c r="H28" t="n">
+        <v>12.2</v>
       </c>
     </row>
     <row r="29">
@@ -1460,22 +1547,25 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Jun-10-2026</t>
+          <t>May-22-2026</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>50.9</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>113.7 t</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>137.6</v>
+        <v>160</v>
+      </c>
+      <c r="E29" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>191.4 t</t>
+        </is>
       </c>
       <c r="G29" t="n">
-        <v>15.9</v>
+        <v>103.9</v>
+      </c>
+      <c r="H29" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="30">
@@ -1491,22 +1581,25 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>05-11-2026</t>
+          <t>05-04-2026</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>186.1 t</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>125.3</v>
+        <v>160</v>
+      </c>
+      <c r="E30" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>268.5 t</t>
+        </is>
       </c>
       <c r="G30" t="n">
-        <v>12.5</v>
+        <v>106.3</v>
+      </c>
+      <c r="H30" t="n">
+        <v>15.7</v>
       </c>
     </row>
     <row r="31">
@@ -1522,21 +1615,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>70.8</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>241.3 t</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>0.126</v>
+        <v>160</v>
+      </c>
+      <c r="E31" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>237.8 t</t>
+        </is>
       </c>
       <c r="G31" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="H31" t="n">
         <v>9999</v>
       </c>
     </row>
@@ -1553,22 +1649,25 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026/06/13</t>
+          <t>2026/05/21</t>
         </is>
       </c>
       <c r="D32" t="n">
+        <v>120</v>
+      </c>
+      <c r="E32" t="n">
         <v>-99</v>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>115.9 t</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>123.1</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>189.5 t</t>
+        </is>
       </c>
       <c r="G32" t="n">
-        <v>15.2</v>
+        <v>123.2</v>
+      </c>
+      <c r="H32" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="33">
@@ -1584,22 +1683,25 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>May-26-2026</t>
+          <t>May-15-2026</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>208.4 t</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>95.7</v>
+        <v>120</v>
+      </c>
+      <c r="E33" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>195.9 t</t>
+        </is>
       </c>
       <c r="G33" t="n">
-        <v>16.1</v>
+        <v>100.1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>15.4</v>
       </c>
     </row>
     <row r="34">
@@ -1615,22 +1717,25 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>05-25-2026</t>
+          <t>05-15-2026</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>158.9 t</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>0.135</v>
+        <v>240</v>
+      </c>
+      <c r="E34" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>386.2 t</t>
+        </is>
       </c>
       <c r="G34" t="n">
-        <v>16.4</v>
+        <v>0.08</v>
+      </c>
+      <c r="H34" t="n">
+        <v>15.4</v>
       </c>
     </row>
     <row r="35">
@@ -1646,22 +1751,25 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>60.6</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>122.2 t</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>123.4</v>
+        <v>120</v>
+      </c>
+      <c r="E35" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>185.9 t</t>
+        </is>
       </c>
       <c r="G35" t="n">
-        <v>12.5</v>
+        <v>131.3</v>
+      </c>
+      <c r="H35" t="n">
+        <v>14.7</v>
       </c>
     </row>
     <row r="36">
@@ -1677,22 +1785,25 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026/05/21</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>55.3</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>115.2 t</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>86</v>
+        <v>160</v>
+      </c>
+      <c r="E36" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>215.8 t</t>
+        </is>
       </c>
       <c r="G36" t="n">
-        <v>12.4</v>
+        <v>89.40000000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>11.7</v>
       </c>
     </row>
     <row r="37">
@@ -1712,17 +1823,20 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>55.7</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>148.7 t</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>0.08500000000000001</v>
+        <v>160</v>
+      </c>
+      <c r="E37" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>255.6 t</t>
+        </is>
       </c>
       <c r="G37" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H37" t="n">
         <v>12.9</v>
       </c>
     </row>
@@ -1739,22 +1853,25 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>May-07-2026</t>
+          <t>May-17-2026</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>182.9 t</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>0.127</v>
+        <v>240</v>
+      </c>
+      <c r="E38" t="n">
+        <v>62</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>402.2 t</t>
+        </is>
       </c>
       <c r="G38" t="n">
-        <v>13.3</v>
+        <v>0.103</v>
+      </c>
+      <c r="H38" t="n">
+        <v>13.5</v>
       </c>
     </row>
     <row r="39">
@@ -1770,22 +1887,25 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026/05/13</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>60</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>206.4 t</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>0.129</v>
+        <v>80</v>
+      </c>
+      <c r="E39" t="n">
+        <v>54</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>120.3 t</t>
+        </is>
       </c>
       <c r="G39" t="n">
-        <v>15.6</v>
+        <v>0.13</v>
+      </c>
+      <c r="H39" t="n">
+        <v>12.2</v>
       </c>
     </row>
     <row r="41">
@@ -1806,14 +1926,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1824,20 +1945,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Acres</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Yield (bu/ac)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>harvest weight</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>N rate</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Moisture %</t>
         </is>
@@ -1865,6 +1991,10 @@
         <f>COUNT(Data!G2:G39)</f>
         <v/>
       </c>
+      <c r="F2">
+        <f>COUNT(Data!H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1888,6 +2018,10 @@
         <f>COUNTA(Data!G2:G39)</f>
         <v/>
       </c>
+      <c r="F3">
+        <f>COUNTA(Data!H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1911,6 +2045,10 @@
         <f>MIN(Data!G2:G39)</f>
         <v/>
       </c>
+      <c r="F4">
+        <f>MIN(Data!H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1934,6 +2072,10 @@
         <f>MAX(Data!G2:G39)</f>
         <v/>
       </c>
+      <c r="F5">
+        <f>MAX(Data!H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1957,6 +2099,10 @@
         <f>AVERAGE(Data!G2:G39)</f>
         <v/>
       </c>
+      <c r="F6">
+        <f>AVERAGE(Data!H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1978,6 +2124,10 @@
       </c>
       <c r="E7">
         <f>MEDIAN(Data!G2:G39)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>MEDIAN(Data!H2:H39)</f>
         <v/>
       </c>
     </row>
@@ -2120,17 +2270,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2151,25 +2302,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>acres</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>yield_bu_ac</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>weight_t</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>n_rate_kg_ha</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>moisture_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>duplicate_flag</t>
         </is>
@@ -2189,22 +2345,26 @@
         <v/>
       </c>
       <c r="D2">
-        <f>IF(OR(Data!D2=-99,Data!D2&lt;0,Data!D2&gt;200),"",Data!D2)</f>
+        <f>Data!D2</f>
         <v/>
       </c>
       <c r="E2">
-        <f>VALUE(SUBSTITUTE(Data!E2," t",""))</f>
+        <f>IF(OR(Data!E2=-99,Data!E2&lt;0,Data!E2&gt;200),"",Data!E2)</f>
         <v/>
       </c>
       <c r="F2">
-        <f>IF(Data!F2&lt;1,Data!F2*1000,Data!F2)</f>
+        <f>VALUE(SUBSTITUTE(Data!F2," t",""))</f>
         <v/>
       </c>
       <c r="G2">
-        <f>IF(OR(Data!G2="N/A",Data!G2="missing",Data!G2="",Data!G2=9999),"",Data!G2)</f>
+        <f>IF(Data!G2&lt;1,Data!G2*1000,Data!G2)</f>
         <v/>
       </c>
       <c r="H2">
+        <f>IF(OR(Data!H2="N/A",Data!H2="missing",Data!H2="",Data!H2=9999),"",Data!H2)</f>
+        <v/>
+      </c>
+      <c r="I2">
         <f>COUNTIF(Data!$A$2:$A2,Data!A2)&gt;1</f>
         <v/>
       </c>
@@ -2223,22 +2383,26 @@
         <v/>
       </c>
       <c r="D3">
-        <f>IF(OR(Data!D3=-99,Data!D3&lt;0,Data!D3&gt;200),"",Data!D3)</f>
+        <f>Data!D3</f>
         <v/>
       </c>
       <c r="E3">
-        <f>VALUE(SUBSTITUTE(Data!E3," t",""))</f>
+        <f>IF(OR(Data!E3=-99,Data!E3&lt;0,Data!E3&gt;200),"",Data!E3)</f>
         <v/>
       </c>
       <c r="F3">
-        <f>IF(Data!F3&lt;1,Data!F3*1000,Data!F3)</f>
+        <f>VALUE(SUBSTITUTE(Data!F3," t",""))</f>
         <v/>
       </c>
       <c r="G3">
-        <f>IF(OR(Data!G3="N/A",Data!G3="missing",Data!G3="",Data!G3=9999),"",Data!G3)</f>
+        <f>IF(Data!G3&lt;1,Data!G3*1000,Data!G3)</f>
         <v/>
       </c>
       <c r="H3">
+        <f>IF(OR(Data!H3="N/A",Data!H3="missing",Data!H3="",Data!H3=9999),"",Data!H3)</f>
+        <v/>
+      </c>
+      <c r="I3">
         <f>COUNTIF(Data!$A$2:$A3,Data!A3)&gt;1</f>
         <v/>
       </c>
@@ -2257,22 +2421,26 @@
         <v/>
       </c>
       <c r="D4">
-        <f>IF(OR(Data!D4=-99,Data!D4&lt;0,Data!D4&gt;200),"",Data!D4)</f>
+        <f>Data!D4</f>
         <v/>
       </c>
       <c r="E4">
-        <f>VALUE(SUBSTITUTE(Data!E4," t",""))</f>
+        <f>IF(OR(Data!E4=-99,Data!E4&lt;0,Data!E4&gt;200),"",Data!E4)</f>
         <v/>
       </c>
       <c r="F4">
-        <f>IF(Data!F4&lt;1,Data!F4*1000,Data!F4)</f>
+        <f>VALUE(SUBSTITUTE(Data!F4," t",""))</f>
         <v/>
       </c>
       <c r="G4">
-        <f>IF(OR(Data!G4="N/A",Data!G4="missing",Data!G4="",Data!G4=9999),"",Data!G4)</f>
+        <f>IF(Data!G4&lt;1,Data!G4*1000,Data!G4)</f>
         <v/>
       </c>
       <c r="H4">
+        <f>IF(OR(Data!H4="N/A",Data!H4="missing",Data!H4="",Data!H4=9999),"",Data!H4)</f>
+        <v/>
+      </c>
+      <c r="I4">
         <f>COUNTIF(Data!$A$2:$A4,Data!A4)&gt;1</f>
         <v/>
       </c>
@@ -2291,22 +2459,26 @@
         <v/>
       </c>
       <c r="D5">
-        <f>IF(OR(Data!D5=-99,Data!D5&lt;0,Data!D5&gt;200),"",Data!D5)</f>
+        <f>Data!D5</f>
         <v/>
       </c>
       <c r="E5">
-        <f>VALUE(SUBSTITUTE(Data!E5," t",""))</f>
+        <f>IF(OR(Data!E5=-99,Data!E5&lt;0,Data!E5&gt;200),"",Data!E5)</f>
         <v/>
       </c>
       <c r="F5">
-        <f>IF(Data!F5&lt;1,Data!F5*1000,Data!F5)</f>
+        <f>VALUE(SUBSTITUTE(Data!F5," t",""))</f>
         <v/>
       </c>
       <c r="G5">
-        <f>IF(OR(Data!G5="N/A",Data!G5="missing",Data!G5="",Data!G5=9999),"",Data!G5)</f>
+        <f>IF(Data!G5&lt;1,Data!G5*1000,Data!G5)</f>
         <v/>
       </c>
       <c r="H5">
+        <f>IF(OR(Data!H5="N/A",Data!H5="missing",Data!H5="",Data!H5=9999),"",Data!H5)</f>
+        <v/>
+      </c>
+      <c r="I5">
         <f>COUNTIF(Data!$A$2:$A5,Data!A5)&gt;1</f>
         <v/>
       </c>
@@ -2325,22 +2497,26 @@
         <v/>
       </c>
       <c r="D6">
-        <f>IF(OR(Data!D6=-99,Data!D6&lt;0,Data!D6&gt;200),"",Data!D6)</f>
+        <f>Data!D6</f>
         <v/>
       </c>
       <c r="E6">
-        <f>VALUE(SUBSTITUTE(Data!E6," t",""))</f>
+        <f>IF(OR(Data!E6=-99,Data!E6&lt;0,Data!E6&gt;200),"",Data!E6)</f>
         <v/>
       </c>
       <c r="F6">
-        <f>IF(Data!F6&lt;1,Data!F6*1000,Data!F6)</f>
+        <f>VALUE(SUBSTITUTE(Data!F6," t",""))</f>
         <v/>
       </c>
       <c r="G6">
-        <f>IF(OR(Data!G6="N/A",Data!G6="missing",Data!G6="",Data!G6=9999),"",Data!G6)</f>
+        <f>IF(Data!G6&lt;1,Data!G6*1000,Data!G6)</f>
         <v/>
       </c>
       <c r="H6">
+        <f>IF(OR(Data!H6="N/A",Data!H6="missing",Data!H6="",Data!H6=9999),"",Data!H6)</f>
+        <v/>
+      </c>
+      <c r="I6">
         <f>COUNTIF(Data!$A$2:$A6,Data!A6)&gt;1</f>
         <v/>
       </c>
@@ -2359,22 +2535,26 @@
         <v/>
       </c>
       <c r="D7">
-        <f>IF(OR(Data!D7=-99,Data!D7&lt;0,Data!D7&gt;200),"",Data!D7)</f>
+        <f>Data!D7</f>
         <v/>
       </c>
       <c r="E7">
-        <f>VALUE(SUBSTITUTE(Data!E7," t",""))</f>
+        <f>IF(OR(Data!E7=-99,Data!E7&lt;0,Data!E7&gt;200),"",Data!E7)</f>
         <v/>
       </c>
       <c r="F7">
-        <f>IF(Data!F7&lt;1,Data!F7*1000,Data!F7)</f>
+        <f>VALUE(SUBSTITUTE(Data!F7," t",""))</f>
         <v/>
       </c>
       <c r="G7">
-        <f>IF(OR(Data!G7="N/A",Data!G7="missing",Data!G7="",Data!G7=9999),"",Data!G7)</f>
+        <f>IF(Data!G7&lt;1,Data!G7*1000,Data!G7)</f>
         <v/>
       </c>
       <c r="H7">
+        <f>IF(OR(Data!H7="N/A",Data!H7="missing",Data!H7="",Data!H7=9999),"",Data!H7)</f>
+        <v/>
+      </c>
+      <c r="I7">
         <f>COUNTIF(Data!$A$2:$A7,Data!A7)&gt;1</f>
         <v/>
       </c>
@@ -2393,22 +2573,26 @@
         <v/>
       </c>
       <c r="D8">
-        <f>IF(OR(Data!D8=-99,Data!D8&lt;0,Data!D8&gt;200),"",Data!D8)</f>
+        <f>Data!D8</f>
         <v/>
       </c>
       <c r="E8">
-        <f>VALUE(SUBSTITUTE(Data!E8," t",""))</f>
+        <f>IF(OR(Data!E8=-99,Data!E8&lt;0,Data!E8&gt;200),"",Data!E8)</f>
         <v/>
       </c>
       <c r="F8">
-        <f>IF(Data!F8&lt;1,Data!F8*1000,Data!F8)</f>
+        <f>VALUE(SUBSTITUTE(Data!F8," t",""))</f>
         <v/>
       </c>
       <c r="G8">
-        <f>IF(OR(Data!G8="N/A",Data!G8="missing",Data!G8="",Data!G8=9999),"",Data!G8)</f>
+        <f>IF(Data!G8&lt;1,Data!G8*1000,Data!G8)</f>
         <v/>
       </c>
       <c r="H8">
+        <f>IF(OR(Data!H8="N/A",Data!H8="missing",Data!H8="",Data!H8=9999),"",Data!H8)</f>
+        <v/>
+      </c>
+      <c r="I8">
         <f>COUNTIF(Data!$A$2:$A8,Data!A8)&gt;1</f>
         <v/>
       </c>
@@ -2427,22 +2611,26 @@
         <v/>
       </c>
       <c r="D9">
-        <f>IF(OR(Data!D9=-99,Data!D9&lt;0,Data!D9&gt;200),"",Data!D9)</f>
+        <f>Data!D9</f>
         <v/>
       </c>
       <c r="E9">
-        <f>VALUE(SUBSTITUTE(Data!E9," t",""))</f>
+        <f>IF(OR(Data!E9=-99,Data!E9&lt;0,Data!E9&gt;200),"",Data!E9)</f>
         <v/>
       </c>
       <c r="F9">
-        <f>IF(Data!F9&lt;1,Data!F9*1000,Data!F9)</f>
+        <f>VALUE(SUBSTITUTE(Data!F9," t",""))</f>
         <v/>
       </c>
       <c r="G9">
-        <f>IF(OR(Data!G9="N/A",Data!G9="missing",Data!G9="",Data!G9=9999),"",Data!G9)</f>
+        <f>IF(Data!G9&lt;1,Data!G9*1000,Data!G9)</f>
         <v/>
       </c>
       <c r="H9">
+        <f>IF(OR(Data!H9="N/A",Data!H9="missing",Data!H9="",Data!H9=9999),"",Data!H9)</f>
+        <v/>
+      </c>
+      <c r="I9">
         <f>COUNTIF(Data!$A$2:$A9,Data!A9)&gt;1</f>
         <v/>
       </c>
@@ -2461,22 +2649,26 @@
         <v/>
       </c>
       <c r="D10">
-        <f>IF(OR(Data!D10=-99,Data!D10&lt;0,Data!D10&gt;200),"",Data!D10)</f>
+        <f>Data!D10</f>
         <v/>
       </c>
       <c r="E10">
-        <f>VALUE(SUBSTITUTE(Data!E10," t",""))</f>
+        <f>IF(OR(Data!E10=-99,Data!E10&lt;0,Data!E10&gt;200),"",Data!E10)</f>
         <v/>
       </c>
       <c r="F10">
-        <f>IF(Data!F10&lt;1,Data!F10*1000,Data!F10)</f>
+        <f>VALUE(SUBSTITUTE(Data!F10," t",""))</f>
         <v/>
       </c>
       <c r="G10">
-        <f>IF(OR(Data!G10="N/A",Data!G10="missing",Data!G10="",Data!G10=9999),"",Data!G10)</f>
+        <f>IF(Data!G10&lt;1,Data!G10*1000,Data!G10)</f>
         <v/>
       </c>
       <c r="H10">
+        <f>IF(OR(Data!H10="N/A",Data!H10="missing",Data!H10="",Data!H10=9999),"",Data!H10)</f>
+        <v/>
+      </c>
+      <c r="I10">
         <f>COUNTIF(Data!$A$2:$A10,Data!A10)&gt;1</f>
         <v/>
       </c>
@@ -2495,22 +2687,26 @@
         <v/>
       </c>
       <c r="D11">
-        <f>IF(OR(Data!D11=-99,Data!D11&lt;0,Data!D11&gt;200),"",Data!D11)</f>
+        <f>Data!D11</f>
         <v/>
       </c>
       <c r="E11">
-        <f>VALUE(SUBSTITUTE(Data!E11," t",""))</f>
+        <f>IF(OR(Data!E11=-99,Data!E11&lt;0,Data!E11&gt;200),"",Data!E11)</f>
         <v/>
       </c>
       <c r="F11">
-        <f>IF(Data!F11&lt;1,Data!F11*1000,Data!F11)</f>
+        <f>VALUE(SUBSTITUTE(Data!F11," t",""))</f>
         <v/>
       </c>
       <c r="G11">
-        <f>IF(OR(Data!G11="N/A",Data!G11="missing",Data!G11="",Data!G11=9999),"",Data!G11)</f>
+        <f>IF(Data!G11&lt;1,Data!G11*1000,Data!G11)</f>
         <v/>
       </c>
       <c r="H11">
+        <f>IF(OR(Data!H11="N/A",Data!H11="missing",Data!H11="",Data!H11=9999),"",Data!H11)</f>
+        <v/>
+      </c>
+      <c r="I11">
         <f>COUNTIF(Data!$A$2:$A11,Data!A11)&gt;1</f>
         <v/>
       </c>
@@ -2529,22 +2725,26 @@
         <v/>
       </c>
       <c r="D12">
-        <f>IF(OR(Data!D12=-99,Data!D12&lt;0,Data!D12&gt;200),"",Data!D12)</f>
+        <f>Data!D12</f>
         <v/>
       </c>
       <c r="E12">
-        <f>VALUE(SUBSTITUTE(Data!E12," t",""))</f>
+        <f>IF(OR(Data!E12=-99,Data!E12&lt;0,Data!E12&gt;200),"",Data!E12)</f>
         <v/>
       </c>
       <c r="F12">
-        <f>IF(Data!F12&lt;1,Data!F12*1000,Data!F12)</f>
+        <f>VALUE(SUBSTITUTE(Data!F12," t",""))</f>
         <v/>
       </c>
       <c r="G12">
-        <f>IF(OR(Data!G12="N/A",Data!G12="missing",Data!G12="",Data!G12=9999),"",Data!G12)</f>
+        <f>IF(Data!G12&lt;1,Data!G12*1000,Data!G12)</f>
         <v/>
       </c>
       <c r="H12">
+        <f>IF(OR(Data!H12="N/A",Data!H12="missing",Data!H12="",Data!H12=9999),"",Data!H12)</f>
+        <v/>
+      </c>
+      <c r="I12">
         <f>COUNTIF(Data!$A$2:$A12,Data!A12)&gt;1</f>
         <v/>
       </c>
@@ -2563,22 +2763,26 @@
         <v/>
       </c>
       <c r="D13">
-        <f>IF(OR(Data!D13=-99,Data!D13&lt;0,Data!D13&gt;200),"",Data!D13)</f>
+        <f>Data!D13</f>
         <v/>
       </c>
       <c r="E13">
-        <f>VALUE(SUBSTITUTE(Data!E13," t",""))</f>
+        <f>IF(OR(Data!E13=-99,Data!E13&lt;0,Data!E13&gt;200),"",Data!E13)</f>
         <v/>
       </c>
       <c r="F13">
-        <f>IF(Data!F13&lt;1,Data!F13*1000,Data!F13)</f>
+        <f>VALUE(SUBSTITUTE(Data!F13," t",""))</f>
         <v/>
       </c>
       <c r="G13">
-        <f>IF(OR(Data!G13="N/A",Data!G13="missing",Data!G13="",Data!G13=9999),"",Data!G13)</f>
+        <f>IF(Data!G13&lt;1,Data!G13*1000,Data!G13)</f>
         <v/>
       </c>
       <c r="H13">
+        <f>IF(OR(Data!H13="N/A",Data!H13="missing",Data!H13="",Data!H13=9999),"",Data!H13)</f>
+        <v/>
+      </c>
+      <c r="I13">
         <f>COUNTIF(Data!$A$2:$A13,Data!A13)&gt;1</f>
         <v/>
       </c>
@@ -2597,22 +2801,26 @@
         <v/>
       </c>
       <c r="D14">
-        <f>IF(OR(Data!D14=-99,Data!D14&lt;0,Data!D14&gt;200),"",Data!D14)</f>
+        <f>Data!D14</f>
         <v/>
       </c>
       <c r="E14">
-        <f>VALUE(SUBSTITUTE(Data!E14," t",""))</f>
+        <f>IF(OR(Data!E14=-99,Data!E14&lt;0,Data!E14&gt;200),"",Data!E14)</f>
         <v/>
       </c>
       <c r="F14">
-        <f>IF(Data!F14&lt;1,Data!F14*1000,Data!F14)</f>
+        <f>VALUE(SUBSTITUTE(Data!F14," t",""))</f>
         <v/>
       </c>
       <c r="G14">
-        <f>IF(OR(Data!G14="N/A",Data!G14="missing",Data!G14="",Data!G14=9999),"",Data!G14)</f>
+        <f>IF(Data!G14&lt;1,Data!G14*1000,Data!G14)</f>
         <v/>
       </c>
       <c r="H14">
+        <f>IF(OR(Data!H14="N/A",Data!H14="missing",Data!H14="",Data!H14=9999),"",Data!H14)</f>
+        <v/>
+      </c>
+      <c r="I14">
         <f>COUNTIF(Data!$A$2:$A14,Data!A14)&gt;1</f>
         <v/>
       </c>
@@ -2631,22 +2839,26 @@
         <v/>
       </c>
       <c r="D15">
-        <f>IF(OR(Data!D15=-99,Data!D15&lt;0,Data!D15&gt;200),"",Data!D15)</f>
+        <f>Data!D15</f>
         <v/>
       </c>
       <c r="E15">
-        <f>VALUE(SUBSTITUTE(Data!E15," t",""))</f>
+        <f>IF(OR(Data!E15=-99,Data!E15&lt;0,Data!E15&gt;200),"",Data!E15)</f>
         <v/>
       </c>
       <c r="F15">
-        <f>IF(Data!F15&lt;1,Data!F15*1000,Data!F15)</f>
+        <f>VALUE(SUBSTITUTE(Data!F15," t",""))</f>
         <v/>
       </c>
       <c r="G15">
-        <f>IF(OR(Data!G15="N/A",Data!G15="missing",Data!G15="",Data!G15=9999),"",Data!G15)</f>
+        <f>IF(Data!G15&lt;1,Data!G15*1000,Data!G15)</f>
         <v/>
       </c>
       <c r="H15">
+        <f>IF(OR(Data!H15="N/A",Data!H15="missing",Data!H15="",Data!H15=9999),"",Data!H15)</f>
+        <v/>
+      </c>
+      <c r="I15">
         <f>COUNTIF(Data!$A$2:$A15,Data!A15)&gt;1</f>
         <v/>
       </c>
@@ -2665,22 +2877,26 @@
         <v/>
       </c>
       <c r="D16">
-        <f>IF(OR(Data!D16=-99,Data!D16&lt;0,Data!D16&gt;200),"",Data!D16)</f>
+        <f>Data!D16</f>
         <v/>
       </c>
       <c r="E16">
-        <f>VALUE(SUBSTITUTE(Data!E16," t",""))</f>
+        <f>IF(OR(Data!E16=-99,Data!E16&lt;0,Data!E16&gt;200),"",Data!E16)</f>
         <v/>
       </c>
       <c r="F16">
-        <f>IF(Data!F16&lt;1,Data!F16*1000,Data!F16)</f>
+        <f>VALUE(SUBSTITUTE(Data!F16," t",""))</f>
         <v/>
       </c>
       <c r="G16">
-        <f>IF(OR(Data!G16="N/A",Data!G16="missing",Data!G16="",Data!G16=9999),"",Data!G16)</f>
+        <f>IF(Data!G16&lt;1,Data!G16*1000,Data!G16)</f>
         <v/>
       </c>
       <c r="H16">
+        <f>IF(OR(Data!H16="N/A",Data!H16="missing",Data!H16="",Data!H16=9999),"",Data!H16)</f>
+        <v/>
+      </c>
+      <c r="I16">
         <f>COUNTIF(Data!$A$2:$A16,Data!A16)&gt;1</f>
         <v/>
       </c>
@@ -2699,22 +2915,26 @@
         <v/>
       </c>
       <c r="D17">
-        <f>IF(OR(Data!D17=-99,Data!D17&lt;0,Data!D17&gt;200),"",Data!D17)</f>
+        <f>Data!D17</f>
         <v/>
       </c>
       <c r="E17">
-        <f>VALUE(SUBSTITUTE(Data!E17," t",""))</f>
+        <f>IF(OR(Data!E17=-99,Data!E17&lt;0,Data!E17&gt;200),"",Data!E17)</f>
         <v/>
       </c>
       <c r="F17">
-        <f>IF(Data!F17&lt;1,Data!F17*1000,Data!F17)</f>
+        <f>VALUE(SUBSTITUTE(Data!F17," t",""))</f>
         <v/>
       </c>
       <c r="G17">
-        <f>IF(OR(Data!G17="N/A",Data!G17="missing",Data!G17="",Data!G17=9999),"",Data!G17)</f>
+        <f>IF(Data!G17&lt;1,Data!G17*1000,Data!G17)</f>
         <v/>
       </c>
       <c r="H17">
+        <f>IF(OR(Data!H17="N/A",Data!H17="missing",Data!H17="",Data!H17=9999),"",Data!H17)</f>
+        <v/>
+      </c>
+      <c r="I17">
         <f>COUNTIF(Data!$A$2:$A17,Data!A17)&gt;1</f>
         <v/>
       </c>
@@ -2733,22 +2953,26 @@
         <v/>
       </c>
       <c r="D18">
-        <f>IF(OR(Data!D18=-99,Data!D18&lt;0,Data!D18&gt;200),"",Data!D18)</f>
+        <f>Data!D18</f>
         <v/>
       </c>
       <c r="E18">
-        <f>VALUE(SUBSTITUTE(Data!E18," t",""))</f>
+        <f>IF(OR(Data!E18=-99,Data!E18&lt;0,Data!E18&gt;200),"",Data!E18)</f>
         <v/>
       </c>
       <c r="F18">
-        <f>IF(Data!F18&lt;1,Data!F18*1000,Data!F18)</f>
+        <f>VALUE(SUBSTITUTE(Data!F18," t",""))</f>
         <v/>
       </c>
       <c r="G18">
-        <f>IF(OR(Data!G18="N/A",Data!G18="missing",Data!G18="",Data!G18=9999),"",Data!G18)</f>
+        <f>IF(Data!G18&lt;1,Data!G18*1000,Data!G18)</f>
         <v/>
       </c>
       <c r="H18">
+        <f>IF(OR(Data!H18="N/A",Data!H18="missing",Data!H18="",Data!H18=9999),"",Data!H18)</f>
+        <v/>
+      </c>
+      <c r="I18">
         <f>COUNTIF(Data!$A$2:$A18,Data!A18)&gt;1</f>
         <v/>
       </c>
@@ -2767,22 +2991,26 @@
         <v/>
       </c>
       <c r="D19">
-        <f>IF(OR(Data!D19=-99,Data!D19&lt;0,Data!D19&gt;200),"",Data!D19)</f>
+        <f>Data!D19</f>
         <v/>
       </c>
       <c r="E19">
-        <f>VALUE(SUBSTITUTE(Data!E19," t",""))</f>
+        <f>IF(OR(Data!E19=-99,Data!E19&lt;0,Data!E19&gt;200),"",Data!E19)</f>
         <v/>
       </c>
       <c r="F19">
-        <f>IF(Data!F19&lt;1,Data!F19*1000,Data!F19)</f>
+        <f>VALUE(SUBSTITUTE(Data!F19," t",""))</f>
         <v/>
       </c>
       <c r="G19">
-        <f>IF(OR(Data!G19="N/A",Data!G19="missing",Data!G19="",Data!G19=9999),"",Data!G19)</f>
+        <f>IF(Data!G19&lt;1,Data!G19*1000,Data!G19)</f>
         <v/>
       </c>
       <c r="H19">
+        <f>IF(OR(Data!H19="N/A",Data!H19="missing",Data!H19="",Data!H19=9999),"",Data!H19)</f>
+        <v/>
+      </c>
+      <c r="I19">
         <f>COUNTIF(Data!$A$2:$A19,Data!A19)&gt;1</f>
         <v/>
       </c>
@@ -2801,22 +3029,26 @@
         <v/>
       </c>
       <c r="D20">
-        <f>IF(OR(Data!D20=-99,Data!D20&lt;0,Data!D20&gt;200),"",Data!D20)</f>
+        <f>Data!D20</f>
         <v/>
       </c>
       <c r="E20">
-        <f>VALUE(SUBSTITUTE(Data!E20," t",""))</f>
+        <f>IF(OR(Data!E20=-99,Data!E20&lt;0,Data!E20&gt;200),"",Data!E20)</f>
         <v/>
       </c>
       <c r="F20">
-        <f>IF(Data!F20&lt;1,Data!F20*1000,Data!F20)</f>
+        <f>VALUE(SUBSTITUTE(Data!F20," t",""))</f>
         <v/>
       </c>
       <c r="G20">
-        <f>IF(OR(Data!G20="N/A",Data!G20="missing",Data!G20="",Data!G20=9999),"",Data!G20)</f>
+        <f>IF(Data!G20&lt;1,Data!G20*1000,Data!G20)</f>
         <v/>
       </c>
       <c r="H20">
+        <f>IF(OR(Data!H20="N/A",Data!H20="missing",Data!H20="",Data!H20=9999),"",Data!H20)</f>
+        <v/>
+      </c>
+      <c r="I20">
         <f>COUNTIF(Data!$A$2:$A20,Data!A20)&gt;1</f>
         <v/>
       </c>
@@ -2835,22 +3067,26 @@
         <v/>
       </c>
       <c r="D21">
-        <f>IF(OR(Data!D21=-99,Data!D21&lt;0,Data!D21&gt;200),"",Data!D21)</f>
+        <f>Data!D21</f>
         <v/>
       </c>
       <c r="E21">
-        <f>VALUE(SUBSTITUTE(Data!E21," t",""))</f>
+        <f>IF(OR(Data!E21=-99,Data!E21&lt;0,Data!E21&gt;200),"",Data!E21)</f>
         <v/>
       </c>
       <c r="F21">
-        <f>IF(Data!F21&lt;1,Data!F21*1000,Data!F21)</f>
+        <f>VALUE(SUBSTITUTE(Data!F21," t",""))</f>
         <v/>
       </c>
       <c r="G21">
-        <f>IF(OR(Data!G21="N/A",Data!G21="missing",Data!G21="",Data!G21=9999),"",Data!G21)</f>
+        <f>IF(Data!G21&lt;1,Data!G21*1000,Data!G21)</f>
         <v/>
       </c>
       <c r="H21">
+        <f>IF(OR(Data!H21="N/A",Data!H21="missing",Data!H21="",Data!H21=9999),"",Data!H21)</f>
+        <v/>
+      </c>
+      <c r="I21">
         <f>COUNTIF(Data!$A$2:$A21,Data!A21)&gt;1</f>
         <v/>
       </c>
@@ -2869,22 +3105,26 @@
         <v/>
       </c>
       <c r="D22">
-        <f>IF(OR(Data!D22=-99,Data!D22&lt;0,Data!D22&gt;200),"",Data!D22)</f>
+        <f>Data!D22</f>
         <v/>
       </c>
       <c r="E22">
-        <f>VALUE(SUBSTITUTE(Data!E22," t",""))</f>
+        <f>IF(OR(Data!E22=-99,Data!E22&lt;0,Data!E22&gt;200),"",Data!E22)</f>
         <v/>
       </c>
       <c r="F22">
-        <f>IF(Data!F22&lt;1,Data!F22*1000,Data!F22)</f>
+        <f>VALUE(SUBSTITUTE(Data!F22," t",""))</f>
         <v/>
       </c>
       <c r="G22">
-        <f>IF(OR(Data!G22="N/A",Data!G22="missing",Data!G22="",Data!G22=9999),"",Data!G22)</f>
+        <f>IF(Data!G22&lt;1,Data!G22*1000,Data!G22)</f>
         <v/>
       </c>
       <c r="H22">
+        <f>IF(OR(Data!H22="N/A",Data!H22="missing",Data!H22="",Data!H22=9999),"",Data!H22)</f>
+        <v/>
+      </c>
+      <c r="I22">
         <f>COUNTIF(Data!$A$2:$A22,Data!A22)&gt;1</f>
         <v/>
       </c>
@@ -2903,22 +3143,26 @@
         <v/>
       </c>
       <c r="D23">
-        <f>IF(OR(Data!D23=-99,Data!D23&lt;0,Data!D23&gt;200),"",Data!D23)</f>
+        <f>Data!D23</f>
         <v/>
       </c>
       <c r="E23">
-        <f>VALUE(SUBSTITUTE(Data!E23," t",""))</f>
+        <f>IF(OR(Data!E23=-99,Data!E23&lt;0,Data!E23&gt;200),"",Data!E23)</f>
         <v/>
       </c>
       <c r="F23">
-        <f>IF(Data!F23&lt;1,Data!F23*1000,Data!F23)</f>
+        <f>VALUE(SUBSTITUTE(Data!F23," t",""))</f>
         <v/>
       </c>
       <c r="G23">
-        <f>IF(OR(Data!G23="N/A",Data!G23="missing",Data!G23="",Data!G23=9999),"",Data!G23)</f>
+        <f>IF(Data!G23&lt;1,Data!G23*1000,Data!G23)</f>
         <v/>
       </c>
       <c r="H23">
+        <f>IF(OR(Data!H23="N/A",Data!H23="missing",Data!H23="",Data!H23=9999),"",Data!H23)</f>
+        <v/>
+      </c>
+      <c r="I23">
         <f>COUNTIF(Data!$A$2:$A23,Data!A23)&gt;1</f>
         <v/>
       </c>
@@ -2937,22 +3181,26 @@
         <v/>
       </c>
       <c r="D24">
-        <f>IF(OR(Data!D24=-99,Data!D24&lt;0,Data!D24&gt;200),"",Data!D24)</f>
+        <f>Data!D24</f>
         <v/>
       </c>
       <c r="E24">
-        <f>VALUE(SUBSTITUTE(Data!E24," t",""))</f>
+        <f>IF(OR(Data!E24=-99,Data!E24&lt;0,Data!E24&gt;200),"",Data!E24)</f>
         <v/>
       </c>
       <c r="F24">
-        <f>IF(Data!F24&lt;1,Data!F24*1000,Data!F24)</f>
+        <f>VALUE(SUBSTITUTE(Data!F24," t",""))</f>
         <v/>
       </c>
       <c r="G24">
-        <f>IF(OR(Data!G24="N/A",Data!G24="missing",Data!G24="",Data!G24=9999),"",Data!G24)</f>
+        <f>IF(Data!G24&lt;1,Data!G24*1000,Data!G24)</f>
         <v/>
       </c>
       <c r="H24">
+        <f>IF(OR(Data!H24="N/A",Data!H24="missing",Data!H24="",Data!H24=9999),"",Data!H24)</f>
+        <v/>
+      </c>
+      <c r="I24">
         <f>COUNTIF(Data!$A$2:$A24,Data!A24)&gt;1</f>
         <v/>
       </c>
@@ -2971,22 +3219,26 @@
         <v/>
       </c>
       <c r="D25">
-        <f>IF(OR(Data!D25=-99,Data!D25&lt;0,Data!D25&gt;200),"",Data!D25)</f>
+        <f>Data!D25</f>
         <v/>
       </c>
       <c r="E25">
-        <f>VALUE(SUBSTITUTE(Data!E25," t",""))</f>
+        <f>IF(OR(Data!E25=-99,Data!E25&lt;0,Data!E25&gt;200),"",Data!E25)</f>
         <v/>
       </c>
       <c r="F25">
-        <f>IF(Data!F25&lt;1,Data!F25*1000,Data!F25)</f>
+        <f>VALUE(SUBSTITUTE(Data!F25," t",""))</f>
         <v/>
       </c>
       <c r="G25">
-        <f>IF(OR(Data!G25="N/A",Data!G25="missing",Data!G25="",Data!G25=9999),"",Data!G25)</f>
+        <f>IF(Data!G25&lt;1,Data!G25*1000,Data!G25)</f>
         <v/>
       </c>
       <c r="H25">
+        <f>IF(OR(Data!H25="N/A",Data!H25="missing",Data!H25="",Data!H25=9999),"",Data!H25)</f>
+        <v/>
+      </c>
+      <c r="I25">
         <f>COUNTIF(Data!$A$2:$A25,Data!A25)&gt;1</f>
         <v/>
       </c>
@@ -3005,22 +3257,26 @@
         <v/>
       </c>
       <c r="D26">
-        <f>IF(OR(Data!D26=-99,Data!D26&lt;0,Data!D26&gt;200),"",Data!D26)</f>
+        <f>Data!D26</f>
         <v/>
       </c>
       <c r="E26">
-        <f>VALUE(SUBSTITUTE(Data!E26," t",""))</f>
+        <f>IF(OR(Data!E26=-99,Data!E26&lt;0,Data!E26&gt;200),"",Data!E26)</f>
         <v/>
       </c>
       <c r="F26">
-        <f>IF(Data!F26&lt;1,Data!F26*1000,Data!F26)</f>
+        <f>VALUE(SUBSTITUTE(Data!F26," t",""))</f>
         <v/>
       </c>
       <c r="G26">
-        <f>IF(OR(Data!G26="N/A",Data!G26="missing",Data!G26="",Data!G26=9999),"",Data!G26)</f>
+        <f>IF(Data!G26&lt;1,Data!G26*1000,Data!G26)</f>
         <v/>
       </c>
       <c r="H26">
+        <f>IF(OR(Data!H26="N/A",Data!H26="missing",Data!H26="",Data!H26=9999),"",Data!H26)</f>
+        <v/>
+      </c>
+      <c r="I26">
         <f>COUNTIF(Data!$A$2:$A26,Data!A26)&gt;1</f>
         <v/>
       </c>
@@ -3039,22 +3295,26 @@
         <v/>
       </c>
       <c r="D27">
-        <f>IF(OR(Data!D27=-99,Data!D27&lt;0,Data!D27&gt;200),"",Data!D27)</f>
+        <f>Data!D27</f>
         <v/>
       </c>
       <c r="E27">
-        <f>VALUE(SUBSTITUTE(Data!E27," t",""))</f>
+        <f>IF(OR(Data!E27=-99,Data!E27&lt;0,Data!E27&gt;200),"",Data!E27)</f>
         <v/>
       </c>
       <c r="F27">
-        <f>IF(Data!F27&lt;1,Data!F27*1000,Data!F27)</f>
+        <f>VALUE(SUBSTITUTE(Data!F27," t",""))</f>
         <v/>
       </c>
       <c r="G27">
-        <f>IF(OR(Data!G27="N/A",Data!G27="missing",Data!G27="",Data!G27=9999),"",Data!G27)</f>
+        <f>IF(Data!G27&lt;1,Data!G27*1000,Data!G27)</f>
         <v/>
       </c>
       <c r="H27">
+        <f>IF(OR(Data!H27="N/A",Data!H27="missing",Data!H27="",Data!H27=9999),"",Data!H27)</f>
+        <v/>
+      </c>
+      <c r="I27">
         <f>COUNTIF(Data!$A$2:$A27,Data!A27)&gt;1</f>
         <v/>
       </c>
@@ -3073,22 +3333,26 @@
         <v/>
       </c>
       <c r="D28">
-        <f>IF(OR(Data!D28=-99,Data!D28&lt;0,Data!D28&gt;200),"",Data!D28)</f>
+        <f>Data!D28</f>
         <v/>
       </c>
       <c r="E28">
-        <f>VALUE(SUBSTITUTE(Data!E28," t",""))</f>
+        <f>IF(OR(Data!E28=-99,Data!E28&lt;0,Data!E28&gt;200),"",Data!E28)</f>
         <v/>
       </c>
       <c r="F28">
-        <f>IF(Data!F28&lt;1,Data!F28*1000,Data!F28)</f>
+        <f>VALUE(SUBSTITUTE(Data!F28," t",""))</f>
         <v/>
       </c>
       <c r="G28">
-        <f>IF(OR(Data!G28="N/A",Data!G28="missing",Data!G28="",Data!G28=9999),"",Data!G28)</f>
+        <f>IF(Data!G28&lt;1,Data!G28*1000,Data!G28)</f>
         <v/>
       </c>
       <c r="H28">
+        <f>IF(OR(Data!H28="N/A",Data!H28="missing",Data!H28="",Data!H28=9999),"",Data!H28)</f>
+        <v/>
+      </c>
+      <c r="I28">
         <f>COUNTIF(Data!$A$2:$A28,Data!A28)&gt;1</f>
         <v/>
       </c>
@@ -3107,22 +3371,26 @@
         <v/>
       </c>
       <c r="D29">
-        <f>IF(OR(Data!D29=-99,Data!D29&lt;0,Data!D29&gt;200),"",Data!D29)</f>
+        <f>Data!D29</f>
         <v/>
       </c>
       <c r="E29">
-        <f>VALUE(SUBSTITUTE(Data!E29," t",""))</f>
+        <f>IF(OR(Data!E29=-99,Data!E29&lt;0,Data!E29&gt;200),"",Data!E29)</f>
         <v/>
       </c>
       <c r="F29">
-        <f>IF(Data!F29&lt;1,Data!F29*1000,Data!F29)</f>
+        <f>VALUE(SUBSTITUTE(Data!F29," t",""))</f>
         <v/>
       </c>
       <c r="G29">
-        <f>IF(OR(Data!G29="N/A",Data!G29="missing",Data!G29="",Data!G29=9999),"",Data!G29)</f>
+        <f>IF(Data!G29&lt;1,Data!G29*1000,Data!G29)</f>
         <v/>
       </c>
       <c r="H29">
+        <f>IF(OR(Data!H29="N/A",Data!H29="missing",Data!H29="",Data!H29=9999),"",Data!H29)</f>
+        <v/>
+      </c>
+      <c r="I29">
         <f>COUNTIF(Data!$A$2:$A29,Data!A29)&gt;1</f>
         <v/>
       </c>
@@ -3141,22 +3409,26 @@
         <v/>
       </c>
       <c r="D30">
-        <f>IF(OR(Data!D30=-99,Data!D30&lt;0,Data!D30&gt;200),"",Data!D30)</f>
+        <f>Data!D30</f>
         <v/>
       </c>
       <c r="E30">
-        <f>VALUE(SUBSTITUTE(Data!E30," t",""))</f>
+        <f>IF(OR(Data!E30=-99,Data!E30&lt;0,Data!E30&gt;200),"",Data!E30)</f>
         <v/>
       </c>
       <c r="F30">
-        <f>IF(Data!F30&lt;1,Data!F30*1000,Data!F30)</f>
+        <f>VALUE(SUBSTITUTE(Data!F30," t",""))</f>
         <v/>
       </c>
       <c r="G30">
-        <f>IF(OR(Data!G30="N/A",Data!G30="missing",Data!G30="",Data!G30=9999),"",Data!G30)</f>
+        <f>IF(Data!G30&lt;1,Data!G30*1000,Data!G30)</f>
         <v/>
       </c>
       <c r="H30">
+        <f>IF(OR(Data!H30="N/A",Data!H30="missing",Data!H30="",Data!H30=9999),"",Data!H30)</f>
+        <v/>
+      </c>
+      <c r="I30">
         <f>COUNTIF(Data!$A$2:$A30,Data!A30)&gt;1</f>
         <v/>
       </c>
@@ -3175,22 +3447,26 @@
         <v/>
       </c>
       <c r="D31">
-        <f>IF(OR(Data!D31=-99,Data!D31&lt;0,Data!D31&gt;200),"",Data!D31)</f>
+        <f>Data!D31</f>
         <v/>
       </c>
       <c r="E31">
-        <f>VALUE(SUBSTITUTE(Data!E31," t",""))</f>
+        <f>IF(OR(Data!E31=-99,Data!E31&lt;0,Data!E31&gt;200),"",Data!E31)</f>
         <v/>
       </c>
       <c r="F31">
-        <f>IF(Data!F31&lt;1,Data!F31*1000,Data!F31)</f>
+        <f>VALUE(SUBSTITUTE(Data!F31," t",""))</f>
         <v/>
       </c>
       <c r="G31">
-        <f>IF(OR(Data!G31="N/A",Data!G31="missing",Data!G31="",Data!G31=9999),"",Data!G31)</f>
+        <f>IF(Data!G31&lt;1,Data!G31*1000,Data!G31)</f>
         <v/>
       </c>
       <c r="H31">
+        <f>IF(OR(Data!H31="N/A",Data!H31="missing",Data!H31="",Data!H31=9999),"",Data!H31)</f>
+        <v/>
+      </c>
+      <c r="I31">
         <f>COUNTIF(Data!$A$2:$A31,Data!A31)&gt;1</f>
         <v/>
       </c>
@@ -3209,22 +3485,26 @@
         <v/>
       </c>
       <c r="D32">
-        <f>IF(OR(Data!D32=-99,Data!D32&lt;0,Data!D32&gt;200),"",Data!D32)</f>
+        <f>Data!D32</f>
         <v/>
       </c>
       <c r="E32">
-        <f>VALUE(SUBSTITUTE(Data!E32," t",""))</f>
+        <f>IF(OR(Data!E32=-99,Data!E32&lt;0,Data!E32&gt;200),"",Data!E32)</f>
         <v/>
       </c>
       <c r="F32">
-        <f>IF(Data!F32&lt;1,Data!F32*1000,Data!F32)</f>
+        <f>VALUE(SUBSTITUTE(Data!F32," t",""))</f>
         <v/>
       </c>
       <c r="G32">
-        <f>IF(OR(Data!G32="N/A",Data!G32="missing",Data!G32="",Data!G32=9999),"",Data!G32)</f>
+        <f>IF(Data!G32&lt;1,Data!G32*1000,Data!G32)</f>
         <v/>
       </c>
       <c r="H32">
+        <f>IF(OR(Data!H32="N/A",Data!H32="missing",Data!H32="",Data!H32=9999),"",Data!H32)</f>
+        <v/>
+      </c>
+      <c r="I32">
         <f>COUNTIF(Data!$A$2:$A32,Data!A32)&gt;1</f>
         <v/>
       </c>
@@ -3243,22 +3523,26 @@
         <v/>
       </c>
       <c r="D33">
-        <f>IF(OR(Data!D33=-99,Data!D33&lt;0,Data!D33&gt;200),"",Data!D33)</f>
+        <f>Data!D33</f>
         <v/>
       </c>
       <c r="E33">
-        <f>VALUE(SUBSTITUTE(Data!E33," t",""))</f>
+        <f>IF(OR(Data!E33=-99,Data!E33&lt;0,Data!E33&gt;200),"",Data!E33)</f>
         <v/>
       </c>
       <c r="F33">
-        <f>IF(Data!F33&lt;1,Data!F33*1000,Data!F33)</f>
+        <f>VALUE(SUBSTITUTE(Data!F33," t",""))</f>
         <v/>
       </c>
       <c r="G33">
-        <f>IF(OR(Data!G33="N/A",Data!G33="missing",Data!G33="",Data!G33=9999),"",Data!G33)</f>
+        <f>IF(Data!G33&lt;1,Data!G33*1000,Data!G33)</f>
         <v/>
       </c>
       <c r="H33">
+        <f>IF(OR(Data!H33="N/A",Data!H33="missing",Data!H33="",Data!H33=9999),"",Data!H33)</f>
+        <v/>
+      </c>
+      <c r="I33">
         <f>COUNTIF(Data!$A$2:$A33,Data!A33)&gt;1</f>
         <v/>
       </c>
@@ -3277,22 +3561,26 @@
         <v/>
       </c>
       <c r="D34">
-        <f>IF(OR(Data!D34=-99,Data!D34&lt;0,Data!D34&gt;200),"",Data!D34)</f>
+        <f>Data!D34</f>
         <v/>
       </c>
       <c r="E34">
-        <f>VALUE(SUBSTITUTE(Data!E34," t",""))</f>
+        <f>IF(OR(Data!E34=-99,Data!E34&lt;0,Data!E34&gt;200),"",Data!E34)</f>
         <v/>
       </c>
       <c r="F34">
-        <f>IF(Data!F34&lt;1,Data!F34*1000,Data!F34)</f>
+        <f>VALUE(SUBSTITUTE(Data!F34," t",""))</f>
         <v/>
       </c>
       <c r="G34">
-        <f>IF(OR(Data!G34="N/A",Data!G34="missing",Data!G34="",Data!G34=9999),"",Data!G34)</f>
+        <f>IF(Data!G34&lt;1,Data!G34*1000,Data!G34)</f>
         <v/>
       </c>
       <c r="H34">
+        <f>IF(OR(Data!H34="N/A",Data!H34="missing",Data!H34="",Data!H34=9999),"",Data!H34)</f>
+        <v/>
+      </c>
+      <c r="I34">
         <f>COUNTIF(Data!$A$2:$A34,Data!A34)&gt;1</f>
         <v/>
       </c>
@@ -3311,22 +3599,26 @@
         <v/>
       </c>
       <c r="D35">
-        <f>IF(OR(Data!D35=-99,Data!D35&lt;0,Data!D35&gt;200),"",Data!D35)</f>
+        <f>Data!D35</f>
         <v/>
       </c>
       <c r="E35">
-        <f>VALUE(SUBSTITUTE(Data!E35," t",""))</f>
+        <f>IF(OR(Data!E35=-99,Data!E35&lt;0,Data!E35&gt;200),"",Data!E35)</f>
         <v/>
       </c>
       <c r="F35">
-        <f>IF(Data!F35&lt;1,Data!F35*1000,Data!F35)</f>
+        <f>VALUE(SUBSTITUTE(Data!F35," t",""))</f>
         <v/>
       </c>
       <c r="G35">
-        <f>IF(OR(Data!G35="N/A",Data!G35="missing",Data!G35="",Data!G35=9999),"",Data!G35)</f>
+        <f>IF(Data!G35&lt;1,Data!G35*1000,Data!G35)</f>
         <v/>
       </c>
       <c r="H35">
+        <f>IF(OR(Data!H35="N/A",Data!H35="missing",Data!H35="",Data!H35=9999),"",Data!H35)</f>
+        <v/>
+      </c>
+      <c r="I35">
         <f>COUNTIF(Data!$A$2:$A35,Data!A35)&gt;1</f>
         <v/>
       </c>
@@ -3345,22 +3637,26 @@
         <v/>
       </c>
       <c r="D36">
-        <f>IF(OR(Data!D36=-99,Data!D36&lt;0,Data!D36&gt;200),"",Data!D36)</f>
+        <f>Data!D36</f>
         <v/>
       </c>
       <c r="E36">
-        <f>VALUE(SUBSTITUTE(Data!E36," t",""))</f>
+        <f>IF(OR(Data!E36=-99,Data!E36&lt;0,Data!E36&gt;200),"",Data!E36)</f>
         <v/>
       </c>
       <c r="F36">
-        <f>IF(Data!F36&lt;1,Data!F36*1000,Data!F36)</f>
+        <f>VALUE(SUBSTITUTE(Data!F36," t",""))</f>
         <v/>
       </c>
       <c r="G36">
-        <f>IF(OR(Data!G36="N/A",Data!G36="missing",Data!G36="",Data!G36=9999),"",Data!G36)</f>
+        <f>IF(Data!G36&lt;1,Data!G36*1000,Data!G36)</f>
         <v/>
       </c>
       <c r="H36">
+        <f>IF(OR(Data!H36="N/A",Data!H36="missing",Data!H36="",Data!H36=9999),"",Data!H36)</f>
+        <v/>
+      </c>
+      <c r="I36">
         <f>COUNTIF(Data!$A$2:$A36,Data!A36)&gt;1</f>
         <v/>
       </c>
@@ -3379,22 +3675,26 @@
         <v/>
       </c>
       <c r="D37">
-        <f>IF(OR(Data!D37=-99,Data!D37&lt;0,Data!D37&gt;200),"",Data!D37)</f>
+        <f>Data!D37</f>
         <v/>
       </c>
       <c r="E37">
-        <f>VALUE(SUBSTITUTE(Data!E37," t",""))</f>
+        <f>IF(OR(Data!E37=-99,Data!E37&lt;0,Data!E37&gt;200),"",Data!E37)</f>
         <v/>
       </c>
       <c r="F37">
-        <f>IF(Data!F37&lt;1,Data!F37*1000,Data!F37)</f>
+        <f>VALUE(SUBSTITUTE(Data!F37," t",""))</f>
         <v/>
       </c>
       <c r="G37">
-        <f>IF(OR(Data!G37="N/A",Data!G37="missing",Data!G37="",Data!G37=9999),"",Data!G37)</f>
+        <f>IF(Data!G37&lt;1,Data!G37*1000,Data!G37)</f>
         <v/>
       </c>
       <c r="H37">
+        <f>IF(OR(Data!H37="N/A",Data!H37="missing",Data!H37="",Data!H37=9999),"",Data!H37)</f>
+        <v/>
+      </c>
+      <c r="I37">
         <f>COUNTIF(Data!$A$2:$A37,Data!A37)&gt;1</f>
         <v/>
       </c>
@@ -3413,22 +3713,26 @@
         <v/>
       </c>
       <c r="D38">
-        <f>IF(OR(Data!D38=-99,Data!D38&lt;0,Data!D38&gt;200),"",Data!D38)</f>
+        <f>Data!D38</f>
         <v/>
       </c>
       <c r="E38">
-        <f>VALUE(SUBSTITUTE(Data!E38," t",""))</f>
+        <f>IF(OR(Data!E38=-99,Data!E38&lt;0,Data!E38&gt;200),"",Data!E38)</f>
         <v/>
       </c>
       <c r="F38">
-        <f>IF(Data!F38&lt;1,Data!F38*1000,Data!F38)</f>
+        <f>VALUE(SUBSTITUTE(Data!F38," t",""))</f>
         <v/>
       </c>
       <c r="G38">
-        <f>IF(OR(Data!G38="N/A",Data!G38="missing",Data!G38="",Data!G38=9999),"",Data!G38)</f>
+        <f>IF(Data!G38&lt;1,Data!G38*1000,Data!G38)</f>
         <v/>
       </c>
       <c r="H38">
+        <f>IF(OR(Data!H38="N/A",Data!H38="missing",Data!H38="",Data!H38=9999),"",Data!H38)</f>
+        <v/>
+      </c>
+      <c r="I38">
         <f>COUNTIF(Data!$A$2:$A38,Data!A38)&gt;1</f>
         <v/>
       </c>
@@ -3447,22 +3751,26 @@
         <v/>
       </c>
       <c r="D39">
-        <f>IF(OR(Data!D39=-99,Data!D39&lt;0,Data!D39&gt;200),"",Data!D39)</f>
+        <f>Data!D39</f>
         <v/>
       </c>
       <c r="E39">
-        <f>VALUE(SUBSTITUTE(Data!E39," t",""))</f>
+        <f>IF(OR(Data!E39=-99,Data!E39&lt;0,Data!E39&gt;200),"",Data!E39)</f>
         <v/>
       </c>
       <c r="F39">
-        <f>IF(Data!F39&lt;1,Data!F39*1000,Data!F39)</f>
+        <f>VALUE(SUBSTITUTE(Data!F39," t",""))</f>
         <v/>
       </c>
       <c r="G39">
-        <f>IF(OR(Data!G39="N/A",Data!G39="missing",Data!G39="",Data!G39=9999),"",Data!G39)</f>
+        <f>IF(Data!G39&lt;1,Data!G39*1000,Data!G39)</f>
         <v/>
       </c>
       <c r="H39">
+        <f>IF(OR(Data!H39="N/A",Data!H39="missing",Data!H39="",Data!H39=9999),"",Data!H39)</f>
+        <v/>
+      </c>
+      <c r="I39">
         <f>COUNTIF(Data!$A$2:$A39,Data!A39)&gt;1</f>
         <v/>
       </c>
@@ -3480,18 +3788,18 @@
           <t>Minimum</t>
         </is>
       </c>
-      <c r="D42">
-        <f>MIN(D2:D39)</f>
-        <v/>
-      </c>
-      <c r="F42">
-        <f>MIN(F2:F39)</f>
+      <c r="E42">
+        <f>MIN(E2:E39)</f>
         <v/>
       </c>
       <c r="G42">
         <f>MIN(G2:G39)</f>
         <v/>
       </c>
+      <c r="H42">
+        <f>MIN(H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3499,18 +3807,18 @@
           <t>Maximum</t>
         </is>
       </c>
-      <c r="D43">
-        <f>MAX(D2:D39)</f>
-        <v/>
-      </c>
-      <c r="F43">
-        <f>MAX(F2:F39)</f>
+      <c r="E43">
+        <f>MAX(E2:E39)</f>
         <v/>
       </c>
       <c r="G43">
         <f>MAX(G2:G39)</f>
         <v/>
       </c>
+      <c r="H43">
+        <f>MAX(H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3518,18 +3826,18 @@
           <t>Mean</t>
         </is>
       </c>
-      <c r="D44">
-        <f>AVERAGE(D2:D39)</f>
-        <v/>
-      </c>
-      <c r="F44">
-        <f>AVERAGE(F2:F39)</f>
+      <c r="E44">
+        <f>AVERAGE(E2:E39)</f>
         <v/>
       </c>
       <c r="G44">
         <f>AVERAGE(G2:G39)</f>
         <v/>
       </c>
+      <c r="H44">
+        <f>AVERAGE(H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3537,18 +3845,18 @@
           <t>Median</t>
         </is>
       </c>
-      <c r="D45">
-        <f>MEDIAN(D2:D39)</f>
-        <v/>
-      </c>
-      <c r="F45">
-        <f>MEDIAN(F2:F39)</f>
+      <c r="E45">
+        <f>MEDIAN(E2:E39)</f>
         <v/>
       </c>
       <c r="G45">
         <f>MEDIAN(G2:G39)</f>
         <v/>
       </c>
+      <c r="H45">
+        <f>MEDIAN(H2:H39)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3580,6 +3888,13 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>A consistency check the columns now support: weight_t should be close to yield_bu_ac x acres x 0.02722. Rows that fail it deserve a second look.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>duplicate_flag: TRUE marks the second appearance of a field ID. Filter on TRUE and delete those rows when saving a final copy.</t>
         </is>

</xml_diff>

<commit_message>
Duplicates moved into the first eight rows; chapter, workbook regenerated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod03_field_records_cleaning.xlsx
+++ b/textbook_examples/mod03_field_records_cleaning.xlsx
@@ -509,7 +509,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Duplicate rows              -- counted on Checks; flagged in Clean column I</t>
+          <t xml:space="preserve">  3. Duplicate rows              -- F002 and F005 appear twice; counted on Checks, flagged in Clean column I</t>
         </is>
       </c>
     </row>
@@ -719,247 +719,247 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>F004</t>
+          <t>F002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Brandon AAC</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jun-18-2026</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>320</v>
       </c>
       <c r="E5" t="n">
-        <v>-99</v>
+        <v>54.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>642.5 t</t>
+          <t>476.0 t</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>116.7</v>
+        <v>96.2</v>
       </c>
       <c r="H5" t="n">
-        <v>15.4</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F005</t>
+          <t>F004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>Brandon AAC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>06-06-2026</t>
+          <t>Jun-18-2026</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>320</v>
       </c>
       <c r="E6" t="n">
-        <v>65.8</v>
+        <v>-99</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>561.5 t</t>
+          <t>642.5 t</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>89.90000000000001</v>
+        <v>116.7</v>
       </c>
       <c r="H6" t="n">
-        <v>12.3</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>F006</t>
+          <t>F005</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Brndon</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>06-06-2026</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="E7" t="n">
-        <v>50.8</v>
+        <v>65.8</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>222.8 t</t>
+          <t>561.5 t</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>89.90000000000001</v>
+      </c>
+      <c r="H7" t="n">
+        <v>12.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>F007</t>
+          <t>F006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AAC Viewfield</t>
+          <t>Brndon</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026/06/07</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="E8" t="n">
-        <v>-12</v>
+        <v>50.8</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>138.6 t</t>
+          <t>222.8 t</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>135.9</v>
-      </c>
-      <c r="H8" t="n">
-        <v>14.5</v>
+        <v>0.113</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>F008</t>
+          <t>F005</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AAC Brandon</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>May-18-2026</t>
+          <t>06-06-2026</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="E9" t="n">
-        <v>60.3</v>
+        <v>65.8</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>264.0 t</t>
+          <t>561.5 t</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>127.3</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>F009</t>
+          <t>F007</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>AAC Viewfield</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>05-20-2026</t>
+          <t>2026/06/07</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
-        <v>51.5</v>
+        <v>-12</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>226.5 t</t>
+          <t>138.6 t</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.081</v>
+        <v>135.9</v>
       </c>
       <c r="H10" t="n">
-        <v>13.7</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>F010</t>
+          <t>F008</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Brandon</t>
+          <t>AAC Brandon</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>May-18-2026</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>160</v>
       </c>
       <c r="E11" t="n">
-        <v>58.9</v>
+        <v>60.3</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>256.6 t</t>
+          <t>264.0 t</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>92.40000000000001</v>
+        <v>127.3</v>
       </c>
       <c r="H11" t="n">
-        <v>16.4</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>F011</t>
+          <t>F009</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -969,203 +969,203 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026/05/18</t>
+          <t>05-20-2026</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>320</v>
+        <v>160</v>
       </c>
       <c r="E12" t="n">
-        <v>54.4</v>
+        <v>51.5</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>481.3 t</t>
+          <t>226.5 t</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>82.90000000000001</v>
+        <v>0.081</v>
       </c>
       <c r="H12" t="n">
-        <v>12</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>F012</t>
+          <t>F010</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Brandon AAC</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>May-17-2026</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="E13" t="n">
-        <v>62</v>
+        <v>58.9</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>402.2 t</t>
+          <t>256.6 t</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.103</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>13.5</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>F013</t>
+          <t>F011</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AAC Viewfield</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>05-18-2026</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>240</v>
+        <v>320</v>
       </c>
       <c r="E14" t="n">
-        <v>41.5</v>
+        <v>54.4</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>269.8 t</t>
+          <t>481.3 t</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>82.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>16.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>F014</t>
+          <t>F012</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Brndon</t>
+          <t>Brandon AAC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>May-17-2026</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>160</v>
+        <v>240</v>
       </c>
       <c r="E15" t="n">
-        <v>57.8</v>
+        <v>62</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>249.6 t</t>
+          <t>402.2 t</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>134</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
+        <v>0.103</v>
+      </c>
+      <c r="H15" t="n">
+        <v>13.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>F015</t>
+          <t>F013</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>AAC Viewfield</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>05-18-2026</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>160</v>
+        <v>240</v>
       </c>
       <c r="E16" t="n">
-        <v>54.7</v>
+        <v>41.5</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>234.9 t</t>
+          <t>269.8 t</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.106</v>
+        <v>82.7</v>
       </c>
       <c r="H16" t="n">
-        <v>11.6</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>F016</t>
+          <t>F014</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AAC Brandon</t>
+          <t>Brndon</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>May-17-2026</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>160</v>
       </c>
       <c r="E17" t="n">
-        <v>52.9</v>
+        <v>57.8</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>225.5 t</t>
+          <t>249.6 t</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>128.5</v>
-      </c>
-      <c r="H17" t="n">
-        <v>13</v>
+        <v>134</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>F017</t>
+          <t>F015</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1175,199 +1175,201 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>05-15-2026</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="E18" t="n">
-        <v>63</v>
+        <v>54.7</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>418.7 t</t>
+          <t>234.9 t</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>85.40000000000001</v>
+        <v>0.106</v>
       </c>
       <c r="H18" t="n">
-        <v>15.5</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>F018</t>
+          <t>F016</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Brandon</t>
+          <t>AAC Brandon</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>May-17-2026</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>160</v>
       </c>
       <c r="E19" t="n">
-        <v>63.6</v>
+        <v>52.9</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>283.2 t</t>
+          <t>225.5 t</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.112</v>
+        <v>128.5</v>
       </c>
       <c r="H19" t="n">
-        <v>15.7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>F019</t>
+          <t>F017</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AAC Viewfield</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>05-15-2026</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="E20" t="n">
-        <v>1250</v>
+        <v>63</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>177.8 t</t>
+          <t>418.7 t</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>104.1</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>12.6</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>F020</t>
+          <t>F018</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Brandon AAC</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Jun-11-2026</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>160</v>
       </c>
       <c r="E21" t="n">
-        <v>76.59999999999999</v>
+        <v>63.6</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>323.9 t</t>
+          <t>283.2 t</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>84.7</v>
+        <v>0.112</v>
       </c>
       <c r="H21" t="n">
-        <v>13.1</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>F021</t>
+          <t>F019</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>AAC Viewfield</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>06-10-2026</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="E22" t="n">
-        <v>65.09999999999999</v>
+        <v>1250</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>431.7 t</t>
+          <t>177.8 t</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.129</v>
+        <v>104.1</v>
       </c>
       <c r="H22" t="n">
-        <v>15.4</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>F022</t>
+          <t>F020</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Brndon</t>
+          <t>Brandon AAC</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>Jun-11-2026</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>320</v>
+        <v>160</v>
       </c>
       <c r="E23" t="n">
-        <v>57.5</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>492.0 t</t>
+          <t>323.9 t</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>96.8</v>
-      </c>
-      <c r="H23" t="inlineStr"/>
+        <v>84.7</v>
+      </c>
+      <c r="H23" t="n">
+        <v>13.1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>F023</t>
+          <t>F021</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1377,201 +1379,199 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026/05/09</t>
+          <t>06-10-2026</t>
         </is>
       </c>
       <c r="D24" t="n">
         <v>240</v>
       </c>
       <c r="E24" t="n">
-        <v>-99</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>365.8 t</t>
+          <t>431.7 t</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>87.2</v>
+        <v>0.129</v>
       </c>
       <c r="H24" t="n">
-        <v>16</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>F024</t>
+          <t>F022</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AAC Brandon</t>
+          <t>Brndon</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Jun-26-2026</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="E25" t="n">
-        <v>46.5</v>
+        <v>57.5</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>150.5 t</t>
+          <t>492.0 t</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="H25" t="n">
-        <v>15.3</v>
-      </c>
+        <v>96.8</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>F025</t>
+          <t>F023</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AAC Viewfield</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>06-10-2026</t>
+          <t>2026/05/09</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>160</v>
+        <v>240</v>
       </c>
       <c r="E26" t="n">
-        <v>51.7</v>
+        <v>-99</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>226.1 t</t>
+          <t>365.8 t</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>100.8</v>
+        <v>87.2</v>
       </c>
       <c r="H26" t="n">
-        <v>11.6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>F026</t>
+          <t>F024</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Brandon</t>
+          <t>AAC Brandon</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>Jun-26-2026</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="E27" t="n">
-        <v>59.1</v>
+        <v>46.5</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>252.7 t</t>
+          <t>150.5 t</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>132.9</v>
+        <v>0.124</v>
       </c>
       <c r="H27" t="n">
-        <v>15.7</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>F027</t>
+          <t>F025</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>AAC Viewfield</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>06-10-2026</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="E28" t="n">
-        <v>54</v>
+        <v>51.7</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>120.3 t</t>
+          <t>226.1 t</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.13</v>
+        <v>100.8</v>
       </c>
       <c r="H28" t="n">
-        <v>12.2</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>F028</t>
+          <t>F026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Brandon AAC</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>May-22-2026</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="D29" t="n">
         <v>160</v>
       </c>
       <c r="E29" t="n">
-        <v>43.3</v>
+        <v>59.1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>191.4 t</t>
+          <t>252.7 t</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>103.9</v>
+        <v>132.9</v>
       </c>
       <c r="H29" t="n">
-        <v>15</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>F029</t>
+          <t>F027</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1581,201 +1581,201 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>05-04-2026</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="E30" t="n">
-        <v>63.3</v>
+        <v>54</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>268.5 t</t>
+          <t>120.3 t</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>106.3</v>
+        <v>0.13</v>
       </c>
       <c r="H30" t="n">
-        <v>15.7</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>F030</t>
+          <t>F028</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Brndon</t>
+          <t>Brandon AAC</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>May-22-2026</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>160</v>
       </c>
       <c r="E31" t="n">
-        <v>53.2</v>
+        <v>43.3</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>237.8 t</t>
+          <t>191.4 t</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>0.092</v>
+        <v>103.9</v>
       </c>
       <c r="H31" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>F031</t>
+          <t>F029</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AAC Viewfield</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026/05/21</t>
+          <t>05-04-2026</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="E32" t="n">
-        <v>-99</v>
+        <v>63.3</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>189.5 t</t>
+          <t>268.5 t</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>123.2</v>
+        <v>106.3</v>
       </c>
       <c r="H32" t="n">
-        <v>16</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>F032</t>
+          <t>F030</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AAC Brandon</t>
+          <t>Brndon</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>May-15-2026</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="E33" t="n">
-        <v>60.1</v>
+        <v>53.2</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>195.9 t</t>
+          <t>237.8 t</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>100.1</v>
+        <v>0.092</v>
       </c>
       <c r="H33" t="n">
-        <v>15.4</v>
+        <v>9999</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>F033</t>
+          <t>F031</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>AAC Viewfield</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>05-15-2026</t>
+          <t>2026/05/21</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="E34" t="n">
-        <v>58.6</v>
+        <v>-99</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>386.2 t</t>
+          <t>189.5 t</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.08</v>
+        <v>123.2</v>
       </c>
       <c r="H34" t="n">
-        <v>15.4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>F034</t>
+          <t>F032</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brandon</t>
+          <t>AAC Brandon</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>May-15-2026</t>
         </is>
       </c>
       <c r="D35" t="n">
         <v>120</v>
       </c>
       <c r="E35" t="n">
-        <v>56.8</v>
+        <v>60.1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>185.9 t</t>
+          <t>195.9 t</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>131.3</v>
+        <v>100.1</v>
       </c>
       <c r="H35" t="n">
-        <v>14.7</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>F035</t>
+          <t>F033</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1785,127 +1785,127 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026/05/18</t>
+          <t>05-15-2026</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>160</v>
+        <v>240</v>
       </c>
       <c r="E36" t="n">
-        <v>50.1</v>
+        <v>58.6</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>215.8 t</t>
+          <t>386.2 t</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>89.40000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="H36" t="n">
-        <v>11.7</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>F036</t>
+          <t>F034</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Brandon AAC</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>May-17-2026</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="E37" t="n">
-        <v>58.2</v>
+        <v>56.8</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>255.6 t</t>
+          <t>185.9 t</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>0.13</v>
+        <v>131.3</v>
       </c>
       <c r="H37" t="n">
-        <v>12.9</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>F012</t>
+          <t>F035</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Brandon AAC</t>
+          <t>CDC Landmark</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>May-17-2026</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="E38" t="n">
-        <v>62</v>
+        <v>50.1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>402.2 t</t>
+          <t>215.8 t</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>0.103</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>13.5</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>F027</t>
+          <t>F036</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CDC Landmark</t>
+          <t>Brandon AAC</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>May-17-2026</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="E39" t="n">
-        <v>54</v>
+        <v>58.2</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>120.3 t</t>
+          <t>255.6 t</t>
         </is>
       </c>
       <c r="G39" t="n">
         <v>0.13</v>
       </c>
       <c r="H39" t="n">
-        <v>12.2</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="41">
@@ -3889,7 +3889,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>A consistency check the columns now support: weight_t should be close to yield_bu_ac x acres x 0.02722. Rows that fail it deserve a second look.</t>
+          <t>A consistency check the columns support: weight_t should be close to yield_bu_ac x acres x 0.02722. Rows that fail it deserve a second look.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update cleaning workbook from Excel
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod03_field_records_cleaning.xlsx
+++ b/textbook_examples/mod03_field_records_cleaning.xlsx
@@ -8,27 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="11_F459A3160A9B7F43279732CADF3B43875AA2B4A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD0CA789-9E69-8849-A4F9-5E224104E92F}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="11_F459A3160A9B7F43279732CADF3B43875AA2B4A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4C51E58-28CD-024F-91FF-B70A5964B687}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="RawData" sheetId="2" r:id="rId2"/>
-    <sheet name="DataSummary" sheetId="3" r:id="rId3"/>
+    <sheet name="raw_data" sheetId="2" r:id="rId2"/>
+    <sheet name="data_summary" sheetId="3" r:id="rId3"/>
     <sheet name="clean_data" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">RawData!$H$16:$H$39</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">RawData!$H$1:$H$15</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">RawData!$H$16:$H$39</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">RawData!$H$1:$H$15</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">RawData!$G$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">RawData!$G$2:$G$39</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">RawData!$D$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">RawData!$D$2:$D$39</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">RawData!$E$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">RawData!$E$2:$E$39</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">raw_data!$H$16:$H$39</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">raw_data!$H$1:$H$15</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">raw_data!$H$16:$H$39</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">raw_data!$H$1:$H$15</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">raw_data!$G$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">raw_data!$G$2:$G$39</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">raw_data!$D$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">raw_data!$D$2:$D$39</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">raw_data!$E$1</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">raw_data!$E$2:$E$39</definedName>
     <definedName name="ExternalData_1" localSheetId="3" hidden="1">clean_data!$A$1:$H$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -3821,6 +3821,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{3754D760-2A2C-2B47-AC00-10591B4344D5}">
+  <we:reference id="11d7cf85-ae5a-43b8-bc58-1e1a151cce24" version="1.0.0.1" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;95a756d0-6a79-4d9a-aa9b-500d59265f3c&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A18"/>
@@ -4993,27 +5015,27 @@
         <v>133</v>
       </c>
       <c r="B3" s="13">
-        <f>COUNT(RawData!C2:C39)</f>
+        <f>COUNT(raw_data!C2:C39)</f>
         <v>0</v>
       </c>
       <c r="C3" s="13">
-        <f>COUNT(RawData!D2:D39)</f>
+        <f>COUNT(raw_data!D2:D39)</f>
         <v>38</v>
       </c>
       <c r="D3" s="13">
-        <f>COUNT(RawData!E2:E39)</f>
+        <f>COUNT(raw_data!E2:E39)</f>
         <v>38</v>
       </c>
       <c r="E3" s="13">
-        <f>COUNT(RawData!F2:F39)</f>
+        <f>COUNT(raw_data!F2:F39)</f>
         <v>0</v>
       </c>
       <c r="F3" s="13">
-        <f>COUNT(RawData!G2:G39)</f>
+        <f>COUNT(raw_data!G2:G39)</f>
         <v>38</v>
       </c>
       <c r="G3" s="13">
-        <f>COUNT(RawData!H2:H39)</f>
+        <f>COUNT(raw_data!H2:H39)</f>
         <v>35</v>
       </c>
     </row>
@@ -5022,27 +5044,27 @@
         <v>134</v>
       </c>
       <c r="B4" s="13">
-        <f>COUNTA(RawData!C2:C39)</f>
+        <f>COUNTA(raw_data!C2:C39)</f>
         <v>38</v>
       </c>
       <c r="C4" s="13">
-        <f>COUNTA(RawData!D2:D39)</f>
+        <f>COUNTA(raw_data!D2:D39)</f>
         <v>38</v>
       </c>
       <c r="D4" s="13">
-        <f>COUNTA(RawData!E2:E39)</f>
+        <f>COUNTA(raw_data!E2:E39)</f>
         <v>38</v>
       </c>
       <c r="E4" s="13">
-        <f>COUNTA(RawData!F2:F39)</f>
+        <f>COUNTA(raw_data!F2:F39)</f>
         <v>38</v>
       </c>
       <c r="F4" s="13">
-        <f>COUNTA(RawData!G2:G39)</f>
+        <f>COUNTA(raw_data!G2:G39)</f>
         <v>38</v>
       </c>
       <c r="G4" s="13">
-        <f>COUNTA(RawData!H2:H39)</f>
+        <f>COUNTA(raw_data!H2:H39)</f>
         <v>37</v>
       </c>
     </row>
@@ -5051,27 +5073,27 @@
         <v>135</v>
       </c>
       <c r="B5" s="13">
-        <f>MIN(RawData!C2:C39)</f>
+        <f>MIN(raw_data!C2:C39)</f>
         <v>0</v>
       </c>
       <c r="C5" s="13">
-        <f>MIN(RawData!D2:D39)</f>
+        <f>MIN(raw_data!D2:D39)</f>
         <v>80</v>
       </c>
       <c r="D5" s="13">
-        <f>MIN(RawData!E2:E39)</f>
+        <f>MIN(raw_data!E2:E39)</f>
         <v>-99</v>
       </c>
       <c r="E5" s="13">
-        <f>MIN(RawData!F2:F39)</f>
+        <f>MIN(raw_data!F2:F39)</f>
         <v>0</v>
       </c>
       <c r="F5" s="13">
-        <f>MIN(RawData!G2:G39)</f>
+        <f>MIN(raw_data!G2:G39)</f>
         <v>0.08</v>
       </c>
       <c r="G5" s="13">
-        <f>MIN(RawData!H2:H39)</f>
+        <f>MIN(raw_data!H2:H39)</f>
         <v>11.6</v>
       </c>
     </row>
@@ -5080,27 +5102,27 @@
         <v>136</v>
       </c>
       <c r="B6" s="13">
-        <f>MAX(RawData!C2:C39)</f>
+        <f>MAX(raw_data!C2:C39)</f>
         <v>0</v>
       </c>
       <c r="C6" s="13">
-        <f>MAX(RawData!D2:D39)</f>
+        <f>MAX(raw_data!D2:D39)</f>
         <v>320</v>
       </c>
       <c r="D6" s="13">
-        <f>MAX(RawData!E2:E39)</f>
+        <f>MAX(raw_data!E2:E39)</f>
         <v>1250</v>
       </c>
       <c r="E6" s="13">
-        <f>MAX(RawData!F2:F39)</f>
+        <f>MAX(raw_data!F2:F39)</f>
         <v>0</v>
       </c>
       <c r="F6" s="13">
-        <f>MAX(RawData!G2:G39)</f>
+        <f>MAX(raw_data!G2:G39)</f>
         <v>135.9</v>
       </c>
       <c r="G6" s="13">
-        <f>MAX(RawData!H2:H39)</f>
+        <f>MAX(raw_data!H2:H39)</f>
         <v>9999</v>
       </c>
     </row>
@@ -5109,27 +5131,27 @@
         <v>137</v>
       </c>
       <c r="B7" s="13" t="e">
-        <f>AVERAGE(RawData!C2:C39)</f>
+        <f>AVERAGE(raw_data!C2:C39)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="C7" s="13">
-        <f>AVERAGE(RawData!D2:D39)</f>
+        <f>AVERAGE(raw_data!D2:D39)</f>
         <v>183.15789473684211</v>
       </c>
       <c r="D7" s="13">
-        <f>AVERAGE(RawData!E2:E39)</f>
+        <f>AVERAGE(raw_data!E2:E39)</f>
         <v>74.347368421052622</v>
       </c>
       <c r="E7" s="13" t="e">
-        <f>AVERAGE(RawData!F2:F39)</f>
+        <f>AVERAGE(raw_data!F2:F39)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F7" s="13">
-        <f>AVERAGE(RawData!G2:G39)</f>
+        <f>AVERAGE(raw_data!G2:G39)</f>
         <v>66.610894736842127</v>
       </c>
       <c r="G7" s="13">
-        <f>AVERAGE(RawData!H2:H39)</f>
+        <f>AVERAGE(raw_data!H2:H39)</f>
         <v>299.29428571428576</v>
       </c>
     </row>
@@ -5138,27 +5160,27 @@
         <v>138</v>
       </c>
       <c r="B8" s="13" t="e">
-        <f>MEDIAN(RawData!C2:C39)</f>
+        <f>MEDIAN(raw_data!C2:C39)</f>
         <v>#NUM!</v>
       </c>
       <c r="C8" s="13">
-        <f>MEDIAN(RawData!D2:D39)</f>
+        <f>MEDIAN(raw_data!D2:D39)</f>
         <v>160</v>
       </c>
       <c r="D8" s="13">
-        <f>MEDIAN(RawData!E2:E39)</f>
+        <f>MEDIAN(raw_data!E2:E39)</f>
         <v>55.849999999999994</v>
       </c>
       <c r="E8" s="13" t="e">
-        <f>MEDIAN(RawData!F2:F39)</f>
+        <f>MEDIAN(raw_data!F2:F39)</f>
         <v>#NUM!</v>
       </c>
       <c r="F8" s="13">
-        <f>MEDIAN(RawData!G2:G39)</f>
+        <f>MEDIAN(raw_data!G2:G39)</f>
         <v>88.300000000000011</v>
       </c>
       <c r="G8" s="13">
-        <f>MEDIAN(RawData!H2:H39)</f>
+        <f>MEDIAN(raw_data!H2:H39)</f>
         <v>14.5</v>
       </c>
     </row>
@@ -5178,11 +5200,11 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="str" cm="1">
-        <f t="array" ref="A12:A17">_xlfn.UNIQUE(RawData!B2:B39)</f>
+        <f t="array" ref="A12:A17">_xlfn.UNIQUE(raw_data!B2:B39)</f>
         <v>AAC Viewfield</v>
       </c>
       <c r="B12" s="4">
-        <f>COUNTIF(RawData!B2:B39,A12)</f>
+        <f>COUNTIF(raw_data!B2:B39,A12)</f>
         <v>6</v>
       </c>
     </row>
@@ -5191,7 +5213,7 @@
         <v>Brandon</v>
       </c>
       <c r="B13" s="4">
-        <f>COUNTIF(RawData!B2:B39,A13)</f>
+        <f>COUNTIF(raw_data!B2:B39,A13)</f>
         <v>5</v>
       </c>
     </row>
@@ -5200,7 +5222,7 @@
         <v>CDC Landmark</v>
       </c>
       <c r="B14" s="4">
-        <f>COUNTIF(RawData!B2:B39,A14)</f>
+        <f>COUNTIF(raw_data!B2:B39,A14)</f>
         <v>13</v>
       </c>
     </row>
@@ -5209,7 +5231,7 @@
         <v>Brandon AAC</v>
       </c>
       <c r="B15" s="4">
-        <f>COUNTIF(RawData!B2:B39,A15)</f>
+        <f>COUNTIF(raw_data!B2:B39,A15)</f>
         <v>6</v>
       </c>
     </row>
@@ -5218,7 +5240,7 @@
         <v>Brndon</v>
       </c>
       <c r="B16" s="4">
-        <f>COUNTIF(RawData!B2:B39,A16)</f>
+        <f>COUNTIF(raw_data!B2:B39,A16)</f>
         <v>4</v>
       </c>
     </row>
@@ -5227,7 +5249,7 @@
         <v>AAC Brandon</v>
       </c>
       <c r="B17" s="4">
-        <f>COUNTIF(RawData!B2:B39,A17)</f>
+        <f>COUNTIF(raw_data!B2:B39,A17)</f>
         <v>4</v>
       </c>
     </row>
@@ -5243,7 +5265,7 @@
         <v>141</v>
       </c>
       <c r="B20" s="7">
-        <f>ROWS(RawData!A2:A39)</f>
+        <f>ROWS(raw_data!A2:A39)</f>
         <v>38</v>
       </c>
     </row>
@@ -5252,7 +5274,7 @@
         <v>148</v>
       </c>
       <c r="B21" s="7">
-        <f>ROWS(_xlfn.UNIQUE(RawData!A2:H39))</f>
+        <f>ROWS(_xlfn.UNIQUE(raw_data!A2:H39))</f>
         <v>36</v>
       </c>
     </row>

</xml_diff>